<commit_message>
chore: record coding agent output for issue #5
</commit_message>
<xml_diff>
--- a/workspaces/issue-5/files/監工APP_彙整.xlsx
+++ b/workspaces/issue-5/files/監工APP_彙整.xlsx
@@ -9,7 +9,7 @@
     <sheet name="工作表1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'工作表1'!$A$1:$O$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'工作表1'!$A$1:$P$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,6 +540,9 @@
       <c r="O2" t="n">
         <v>0</v>
       </c>
+      <c r="P2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -596,6 +599,9 @@
       <c r="O3" t="n">
         <v>0</v>
       </c>
+      <c r="P3" t="n">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -653,6 +659,9 @@
       <c r="O4" t="n">
         <v>0</v>
       </c>
+      <c r="P4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -710,6 +719,9 @@
       <c r="O5" t="n">
         <v>0</v>
       </c>
+      <c r="P5" t="n">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -766,6 +778,9 @@
       <c r="O6" t="n">
         <v>0</v>
       </c>
+      <c r="P6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -822,6 +837,9 @@
       <c r="O7" t="n">
         <v>0</v>
       </c>
+      <c r="P7" t="n">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -878,6 +896,9 @@
       <c r="O8" t="n">
         <v>0</v>
       </c>
+      <c r="P8" t="n">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -934,6 +955,9 @@
       <c r="O9" t="n">
         <v>0</v>
       </c>
+      <c r="P9" t="n">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -990,6 +1014,9 @@
       <c r="O10" t="n">
         <v>0</v>
       </c>
+      <c r="P10" t="n">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1046,6 +1073,9 @@
       <c r="O11" t="n">
         <v>0</v>
       </c>
+      <c r="P11" t="n">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1102,6 +1132,9 @@
       <c r="O12" t="n">
         <v>0</v>
       </c>
+      <c r="P12" t="n">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1158,6 +1191,9 @@
       <c r="O13" t="n">
         <v>0</v>
       </c>
+      <c r="P13" t="n">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1214,6 +1250,9 @@
       <c r="O14" t="n">
         <v>0</v>
       </c>
+      <c r="P14" t="n">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1270,6 +1309,9 @@
       <c r="O15" t="n">
         <v>0</v>
       </c>
+      <c r="P15" t="n">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1326,6 +1368,9 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
+      <c r="P16" t="n">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1382,6 +1427,9 @@
       <c r="O17" t="n">
         <v>0</v>
       </c>
+      <c r="P17" t="n">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1438,6 +1486,9 @@
       <c r="O18" t="n">
         <v>0</v>
       </c>
+      <c r="P18" t="n">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1494,6 +1545,9 @@
       <c r="O19" t="n">
         <v>0</v>
       </c>
+      <c r="P19" t="n">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1550,6 +1604,9 @@
       <c r="O20" t="n">
         <v>0</v>
       </c>
+      <c r="P20" t="n">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1606,6 +1663,9 @@
       <c r="O21" t="n">
         <v>0</v>
       </c>
+      <c r="P21" t="n">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1662,6 +1722,9 @@
       <c r="O22" t="n">
         <v>0</v>
       </c>
+      <c r="P22" t="n">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1718,6 +1781,9 @@
       <c r="O23" t="n">
         <v>0</v>
       </c>
+      <c r="P23" t="n">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1774,6 +1840,9 @@
       <c r="O24" t="n">
         <v>0</v>
       </c>
+      <c r="P24" t="n">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1830,6 +1899,9 @@
       <c r="O25" t="n">
         <v>0</v>
       </c>
+      <c r="P25" t="n">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1886,6 +1958,9 @@
       <c r="O26" t="n">
         <v>0</v>
       </c>
+      <c r="P26" t="n">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1942,6 +2017,9 @@
       <c r="O27" t="n">
         <v>0</v>
       </c>
+      <c r="P27" t="n">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1998,6 +2076,9 @@
       <c r="O28" t="n">
         <v>0</v>
       </c>
+      <c r="P28" t="n">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2054,6 +2135,9 @@
       <c r="O29" t="n">
         <v>0</v>
       </c>
+      <c r="P29" t="n">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2110,6 +2194,9 @@
       <c r="O30" t="n">
         <v>0</v>
       </c>
+      <c r="P30" t="n">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2166,6 +2253,9 @@
       <c r="O31" t="n">
         <v>0</v>
       </c>
+      <c r="P31" t="n">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2222,6 +2312,9 @@
       <c r="O32" t="n">
         <v>0</v>
       </c>
+      <c r="P32" t="n">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2278,6 +2371,9 @@
       <c r="O33" t="n">
         <v>0</v>
       </c>
+      <c r="P33" t="n">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2334,6 +2430,9 @@
       <c r="O34" t="n">
         <v>0</v>
       </c>
+      <c r="P34" t="n">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2390,6 +2489,9 @@
       <c r="O35" t="n">
         <v>0</v>
       </c>
+      <c r="P35" t="n">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2446,6 +2548,9 @@
       <c r="O36" t="n">
         <v>0</v>
       </c>
+      <c r="P36" t="n">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2502,6 +2607,9 @@
       <c r="O37" t="n">
         <v>0</v>
       </c>
+      <c r="P37" t="n">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2558,6 +2666,9 @@
       <c r="O38" t="n">
         <v>0</v>
       </c>
+      <c r="P38" t="n">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2614,6 +2725,9 @@
       <c r="O39" t="n">
         <v>0</v>
       </c>
+      <c r="P39" t="n">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2670,6 +2784,9 @@
       <c r="O40" t="n">
         <v>0</v>
       </c>
+      <c r="P40" t="n">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2726,6 +2843,9 @@
       <c r="O41" t="n">
         <v>0</v>
       </c>
+      <c r="P41" t="n">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2782,6 +2902,9 @@
       <c r="O42" t="n">
         <v>0</v>
       </c>
+      <c r="P42" t="n">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2838,6 +2961,9 @@
       <c r="O43" t="n">
         <v>0</v>
       </c>
+      <c r="P43" t="n">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2894,6 +3020,9 @@
       <c r="O44" t="n">
         <v>0</v>
       </c>
+      <c r="P44" t="n">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2950,6 +3079,9 @@
       <c r="O45" t="n">
         <v>0</v>
       </c>
+      <c r="P45" t="n">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3006,6 +3138,9 @@
       <c r="O46" t="n">
         <v>0</v>
       </c>
+      <c r="P46" t="n">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3062,6 +3197,9 @@
       <c r="O47" t="n">
         <v>0</v>
       </c>
+      <c r="P47" t="n">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
@@ -3118,7 +3256,9 @@
       <c r="O48" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P48" s="1" t="n"/>
+      <c r="P48" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -3175,7 +3315,9 @@
       <c r="O49" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P49" s="1" t="n"/>
+      <c r="P49" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
@@ -3232,7 +3374,9 @@
       <c r="O50" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P50" s="1" t="n"/>
+      <c r="P50" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
@@ -3290,7 +3434,9 @@
       <c r="O51" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P51" s="1" t="n"/>
+      <c r="P51" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
@@ -3347,7 +3493,9 @@
       <c r="O52" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P52" s="1" t="n"/>
+      <c r="P52" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
@@ -3404,7 +3552,9 @@
       <c r="O53" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P53" s="1" t="n"/>
+      <c r="P53" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
@@ -3461,7 +3611,9 @@
       <c r="O54" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P54" s="1" t="n"/>
+      <c r="P54" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
@@ -3518,7 +3670,9 @@
       <c r="O55" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P55" s="1" t="n"/>
+      <c r="P55" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
@@ -3575,7 +3729,9 @@
       <c r="O56" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P56" s="1" t="n"/>
+      <c r="P56" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
@@ -3632,7 +3788,9 @@
       <c r="O57" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P57" s="1" t="n"/>
+      <c r="P57" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
@@ -3689,7 +3847,9 @@
       <c r="O58" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P58" s="1" t="n"/>
+      <c r="P58" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
@@ -3746,7 +3906,9 @@
       <c r="O59" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P59" s="1" t="n"/>
+      <c r="P59" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -3804,7 +3966,9 @@
       <c r="O60" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P60" s="1" t="n"/>
+      <c r="P60" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
@@ -3861,7 +4025,9 @@
       <c r="O61" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P61" s="1" t="n"/>
+      <c r="P61" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
@@ -3918,7 +4084,9 @@
       <c r="O62" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P62" s="1" t="n"/>
+      <c r="P62" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
@@ -3976,7 +4144,9 @@
       <c r="O63" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P63" s="1" t="n"/>
+      <c r="P63" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
@@ -4033,7 +4203,9 @@
       <c r="O64" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P64" s="1" t="n"/>
+      <c r="P64" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
@@ -4090,7 +4262,9 @@
       <c r="O65" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P65" s="1" t="n"/>
+      <c r="P65" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
@@ -4148,7 +4322,9 @@
       <c r="O66" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P66" s="1" t="n"/>
+      <c r="P66" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
@@ -4206,7 +4382,9 @@
       <c r="O67" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P67" s="1" t="n"/>
+      <c r="P67" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
@@ -4263,7 +4441,9 @@
       <c r="O68" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P68" s="1" t="n"/>
+      <c r="P68" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
@@ -4320,7 +4500,9 @@
       <c r="O69" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P69" s="1" t="n"/>
+      <c r="P69" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
@@ -4377,7 +4559,9 @@
       <c r="O70" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P70" s="1" t="n"/>
+      <c r="P70" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
@@ -4434,7 +4618,9 @@
       <c r="O71" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P71" s="1" t="n"/>
+      <c r="P71" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
@@ -4492,7 +4678,9 @@
       <c r="O72" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P72" s="1" t="n"/>
+      <c r="P72" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
@@ -4550,7 +4738,9 @@
       <c r="O73" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P73" s="1" t="n"/>
+      <c r="P73" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
@@ -4608,7 +4798,9 @@
       <c r="O74" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P74" s="1" t="n"/>
+      <c r="P74" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
@@ -4665,7 +4857,9 @@
       <c r="O75" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P75" s="1" t="n"/>
+      <c r="P75" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
@@ -4722,7 +4916,9 @@
       <c r="O76" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P76" s="1" t="n"/>
+      <c r="P76" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
@@ -4779,7 +4975,9 @@
       <c r="O77" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P77" s="1" t="n"/>
+      <c r="P77" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
@@ -4837,7 +5035,9 @@
       <c r="O78" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P78" s="1" t="n"/>
+      <c r="P78" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
@@ -4894,7 +5094,9 @@
       <c r="O79" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P79" s="1" t="n"/>
+      <c r="P79" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
@@ -4951,7 +5153,9 @@
       <c r="O80" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P80" s="1" t="n"/>
+      <c r="P80" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
@@ -5008,7 +5212,9 @@
       <c r="O81" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P81" s="1" t="n"/>
+      <c r="P81" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
@@ -5066,7 +5272,9 @@
       <c r="O82" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P82" s="1" t="n"/>
+      <c r="P82" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
@@ -5124,7 +5332,9 @@
       <c r="O83" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P83" s="1" t="n"/>
+      <c r="P83" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
@@ -5181,7 +5391,9 @@
       <c r="O84" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P84" s="1" t="n"/>
+      <c r="P84" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
@@ -5239,7 +5451,9 @@
       <c r="O85" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P85" s="1" t="n"/>
+      <c r="P85" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
@@ -5297,7 +5511,9 @@
       <c r="O86" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P86" s="1" t="n"/>
+      <c r="P86" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
@@ -5355,7 +5571,9 @@
       <c r="O87" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P87" s="1" t="n"/>
+      <c r="P87" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
@@ -5413,7 +5631,9 @@
       <c r="O88" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P88" s="1" t="n"/>
+      <c r="P88" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
@@ -5470,7 +5690,9 @@
       <c r="O89" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P89" s="1" t="n"/>
+      <c r="P89" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
@@ -5530,7 +5752,9 @@
       <c r="O90" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="P90" s="1" t="n"/>
+      <c r="P90" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
@@ -5587,7 +5811,9 @@
       <c r="O91" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P91" s="1" t="n"/>
+      <c r="P91" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
@@ -5645,7 +5871,9 @@
       <c r="O92" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P92" s="1" t="n"/>
+      <c r="P92" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
@@ -5703,7 +5931,9 @@
       <c r="O93" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P93" s="1" t="n"/>
+      <c r="P93" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
@@ -5761,7 +5991,9 @@
       <c r="O94" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P94" s="1" t="n"/>
+      <c r="P94" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
@@ -5819,7 +6051,9 @@
       <c r="O95" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P95" s="1" t="n"/>
+      <c r="P95" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
@@ -5877,7 +6111,9 @@
       <c r="O96" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P96" s="1" t="n"/>
+      <c r="P96" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
@@ -5935,7 +6171,9 @@
       <c r="O97" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P97" s="1" t="n"/>
+      <c r="P97" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
@@ -5993,7 +6231,9 @@
       <c r="O98" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P98" s="1" t="n"/>
+      <c r="P98" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
@@ -6051,7 +6291,9 @@
       <c r="O99" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P99" s="1" t="n"/>
+      <c r="P99" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
@@ -6109,7 +6351,9 @@
       <c r="O100" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P100" s="1" t="n"/>
+      <c r="P100" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
@@ -6167,7 +6411,9 @@
       <c r="O101" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P101" s="1" t="n"/>
+      <c r="P101" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
@@ -6225,7 +6471,9 @@
       <c r="O102" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P102" s="1" t="n"/>
+      <c r="P102" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
@@ -6283,7 +6531,9 @@
       <c r="O103" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P103" s="1" t="n"/>
+      <c r="P103" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
@@ -6341,7 +6591,9 @@
       <c r="O104" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P104" s="1" t="n"/>
+      <c r="P104" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
@@ -6399,7 +6651,9 @@
       <c r="O105" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P105" s="1" t="n"/>
+      <c r="P105" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
@@ -6457,7 +6711,9 @@
       <c r="O106" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P106" s="1" t="n"/>
+      <c r="P106" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
@@ -6515,7 +6771,9 @@
       <c r="O107" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P107" s="1" t="n"/>
+      <c r="P107" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
@@ -6573,7 +6831,9 @@
       <c r="O108" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P108" s="1" t="n"/>
+      <c r="P108" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
@@ -6631,7 +6891,9 @@
       <c r="O109" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P109" s="1" t="n"/>
+      <c r="P109" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
@@ -6689,7 +6951,9 @@
       <c r="O110" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P110" s="1" t="n"/>
+      <c r="P110" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
@@ -6747,7 +7011,9 @@
       <c r="O111" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P111" s="1" t="n"/>
+      <c r="P111" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
@@ -6805,7 +7071,9 @@
       <c r="O112" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P112" s="1" t="n"/>
+      <c r="P112" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
@@ -6863,7 +7131,9 @@
       <c r="O113" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P113" s="1" t="n"/>
+      <c r="P113" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
@@ -6921,7 +7191,9 @@
       <c r="O114" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P114" s="1" t="n"/>
+      <c r="P114" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
@@ -6979,7 +7251,9 @@
       <c r="O115" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P115" s="1" t="n"/>
+      <c r="P115" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
@@ -7037,7 +7311,9 @@
       <c r="O116" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P116" s="1" t="n"/>
+      <c r="P116" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
@@ -7095,7 +7371,9 @@
       <c r="O117" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P117" s="1" t="n"/>
+      <c r="P117" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
@@ -7153,7 +7431,9 @@
       <c r="O118" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P118" s="1" t="n"/>
+      <c r="P118" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
@@ -7211,7 +7491,9 @@
       <c r="O119" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P119" s="1" t="n"/>
+      <c r="P119" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
@@ -7269,7 +7551,9 @@
       <c r="O120" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P120" s="1" t="n"/>
+      <c r="P120" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
@@ -7329,7 +7613,9 @@
       <c r="O121" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P121" s="1" t="n"/>
+      <c r="P121" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
@@ -7387,7 +7673,9 @@
       <c r="O122" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P122" s="1" t="n"/>
+      <c r="P122" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
@@ -7445,7 +7733,9 @@
       <c r="O123" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P123" s="1" t="n"/>
+      <c r="P123" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
@@ -7503,7 +7793,9 @@
       <c r="O124" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P124" s="1" t="n"/>
+      <c r="P124" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
@@ -7561,7 +7853,9 @@
       <c r="O125" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P125" s="1" t="n"/>
+      <c r="P125" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
@@ -7619,7 +7913,9 @@
       <c r="O126" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P126" s="1" t="n"/>
+      <c r="P126" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
@@ -7677,7 +7973,9 @@
       <c r="O127" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P127" s="1" t="n"/>
+      <c r="P127" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
@@ -7735,7 +8033,9 @@
       <c r="O128" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P128" s="1" t="n"/>
+      <c r="P128" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
@@ -7793,7 +8093,9 @@
       <c r="O129" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P129" s="1" t="n"/>
+      <c r="P129" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
@@ -7851,7 +8153,9 @@
       <c r="O130" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P130" s="1" t="n"/>
+      <c r="P130" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
@@ -7909,7 +8213,9 @@
       <c r="O131" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P131" s="1" t="n"/>
+      <c r="P131" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
@@ -7967,7 +8273,9 @@
       <c r="O132" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P132" s="1" t="n"/>
+      <c r="P132" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
@@ -8025,7 +8333,9 @@
       <c r="O133" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P133" s="1" t="n"/>
+      <c r="P133" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
@@ -8083,7 +8393,9 @@
       <c r="O134" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P134" s="1" t="n"/>
+      <c r="P134" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
@@ -8141,7 +8453,9 @@
       <c r="O135" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P135" s="1" t="n"/>
+      <c r="P135" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
@@ -8199,7 +8513,9 @@
       <c r="O136" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P136" s="1" t="n"/>
+      <c r="P136" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
@@ -8257,7 +8573,9 @@
       <c r="O137" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P137" s="1" t="n"/>
+      <c r="P137" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
@@ -8315,7 +8633,9 @@
       <c r="O138" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P138" s="1" t="n"/>
+      <c r="P138" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
@@ -8373,7 +8693,9 @@
       <c r="O139" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P139" s="1" t="n"/>
+      <c r="P139" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
@@ -8433,7 +8755,9 @@
       <c r="O140" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P140" s="1" t="n"/>
+      <c r="P140" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
@@ -8491,7 +8815,9 @@
       <c r="O141" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P141" s="1" t="n"/>
+      <c r="P141" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
@@ -8551,7 +8877,9 @@
       <c r="O142" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P142" s="1" t="n"/>
+      <c r="P142" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
@@ -8609,7 +8937,9 @@
       <c r="O143" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P143" s="1" t="n"/>
+      <c r="P143" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
@@ -8667,7 +8997,9 @@
       <c r="O144" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P144" s="1" t="n"/>
+      <c r="P144" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
@@ -8725,7 +9057,9 @@
       <c r="O145" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P145" s="1" t="n"/>
+      <c r="P145" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
@@ -8783,7 +9117,9 @@
       <c r="O146" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P146" s="1" t="n"/>
+      <c r="P146" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
@@ -8843,7 +9179,9 @@
       <c r="O147" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P147" s="1" t="n"/>
+      <c r="P147" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
@@ -8900,7 +9238,9 @@
       <c r="O148" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P148" s="1" t="n"/>
+      <c r="P148" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
@@ -8958,7 +9298,9 @@
       <c r="O149" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P149" s="1" t="n"/>
+      <c r="P149" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
@@ -9016,7 +9358,9 @@
       <c r="O150" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P150" s="1" t="n"/>
+      <c r="P150" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
@@ -9074,7 +9418,9 @@
       <c r="O151" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P151" s="1" t="n"/>
+      <c r="P151" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
@@ -9132,7 +9478,9 @@
       <c r="O152" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P152" s="1" t="n"/>
+      <c r="P152" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
@@ -9190,7 +9538,9 @@
       <c r="O153" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P153" s="1" t="n"/>
+      <c r="P153" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
@@ -9248,7 +9598,9 @@
       <c r="O154" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P154" s="1" t="n"/>
+      <c r="P154" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
@@ -9306,7 +9658,9 @@
       <c r="O155" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P155" s="1" t="n"/>
+      <c r="P155" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
@@ -9364,7 +9718,9 @@
       <c r="O156" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P156" s="1" t="n"/>
+      <c r="P156" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
@@ -9424,7 +9780,9 @@
       <c r="O157" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P157" s="1" t="n"/>
+      <c r="P157" s="1" t="n">
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n"/>
@@ -14953,7 +15311,7 @@
       <c r="P464" s="1" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O157">
+  <autoFilter ref="A1:P1">
     <sortState ref="A2:P16">
       <sortCondition ref="E1:E16"/>
     </sortState>

</xml_diff>